<commit_message>
update API phieu excel + pdf, up BM phoinapnguoi
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/BM.06-QT.05.11 Bien ban giao nhan phoi nong.xlsx
+++ b/dataproduct.api/wwwroot/templates/BM.06-QT.05.11 Bien ban giao nhan phoi nong.xlsx
@@ -5,22 +5,35 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Software\ThongKePKH\DATAPRODUCT_V2\dataproduct.api\dataproduct.api\wwwroot\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Software\03. ThongKePKH\DATAPRODUCT_V2\dataproduct.api\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65532724-454B-4518-97B1-EEA6B23EE0CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0685331A-0D38-44E2-9CBD-4DEBA07807B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t>BM.06/QT.05.11</t>
   </si>
@@ -117,55 +130,12 @@
     <t>Khối lượng
 (tấn)</t>
   </si>
-  <si>
-    <t>Tổng</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <u/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Lưu ý:</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Tất cả phôi khi đã vào trong nhà máy cán, kể cả còn đang nằm trên bàn con lăn đều bàn giao ngay trong kíp, không để lân sang kíp sau.</t>
-    </r>
-  </si>
-  <si>
-    <t>- Thời điểm xác nhận biên bản giao nhận phôi nóng ở hai thời điểm 8h00p và 20h00p.</t>
-  </si>
-  <si>
-    <t>- Trọng lượng trên được tính theo đơn trọng quy định và chiều dài thực.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  </t>
-  </si>
-  <si>
-    <t>NM.CT DAI</t>
-  </si>
-  <si>
-    <t>P.QLCL</t>
-  </si>
-  <si>
-    <t>NM.HRC1</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <fonts count="14">
     <font>
       <sz val="12"/>
       <name val=".vntime"/>
@@ -239,30 +209,9 @@
       <family val="1"/>
     </font>
     <font>
-      <i/>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <u/>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <b/>
       <i/>
       <sz val="13"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -287,7 +236,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -387,26 +336,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -466,6 +395,19 @@
         <color indexed="64"/>
       </right>
       <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -475,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -488,16 +430,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -508,21 +444,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -542,27 +463,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -579,17 +479,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -601,41 +492,50 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1119,7 +1019,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1138,195 +1038,195 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="4" customFormat="1" ht="20.25" customHeight="1">
-      <c r="L1" s="37"/>
-      <c r="M1" s="38" t="s">
+      <c r="L1" s="23"/>
+      <c r="M1" s="24" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="4" customFormat="1" ht="20.25" customHeight="1">
-      <c r="L2" s="46" t="s">
+      <c r="L2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="46"/>
+      <c r="M2" s="29"/>
     </row>
     <row r="3" spans="1:13" s="4" customFormat="1" ht="20.25" customHeight="1">
       <c r="A3" s="5"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="L3" s="46" t="s">
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="L3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="M3" s="46"/>
-    </row>
-    <row r="4" spans="1:13" s="19" customFormat="1" ht="24" customHeight="1">
-      <c r="A4" s="44" t="s">
+      <c r="M3" s="29"/>
+    </row>
+    <row r="4" spans="1:13" s="12" customFormat="1" ht="24" customHeight="1">
+      <c r="A4" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44"/>
-      <c r="K4" s="44"/>
-      <c r="L4" s="44"/>
-      <c r="M4" s="44"/>
-    </row>
-    <row r="5" spans="1:13" s="12" customFormat="1" ht="24" customHeight="1">
-      <c r="A5" s="44" t="s">
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+    </row>
+    <row r="5" spans="1:13" s="10" customFormat="1" ht="24" customHeight="1">
+      <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="44"/>
-      <c r="J5" s="44"/>
-      <c r="K5" s="44"/>
-      <c r="L5" s="44"/>
-      <c r="M5" s="44"/>
-    </row>
-    <row r="6" spans="1:13" s="40" customFormat="1" ht="18" customHeight="1">
-      <c r="A6" s="45" t="s">
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+    </row>
+    <row r="6" spans="1:13" s="25" customFormat="1" ht="18" customHeight="1">
+      <c r="A6" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="45"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
-      <c r="L6" s="45"/>
-      <c r="M6" s="45"/>
-    </row>
-    <row r="7" spans="1:13" s="9" customFormat="1" ht="18" customHeight="1">
-      <c r="A7" s="43" t="s">
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="28"/>
+      <c r="M6" s="28"/>
+    </row>
+    <row r="7" spans="1:13" s="7" customFormat="1" ht="18" customHeight="1">
+      <c r="A7" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="43"/>
-      <c r="I7" s="43"/>
-      <c r="J7" s="43"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="43"/>
-    </row>
-    <row r="8" spans="1:13" s="22" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A8" s="21" t="s">
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+    </row>
+    <row r="8" spans="1:13" s="15" customFormat="1" ht="17.25" customHeight="1">
+      <c r="A8" s="14" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:13" s="21" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A9" s="22" t="s">
+    <row r="9" spans="1:13" s="14" customFormat="1" ht="19.5" customHeight="1">
+      <c r="A9" s="15" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:13" s="21" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A10" s="22" t="s">
+    <row r="10" spans="1:13" s="14" customFormat="1" ht="19.5" customHeight="1">
+      <c r="A10" s="15" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:13" s="21" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A11" s="22" t="s">
+    <row r="11" spans="1:13" s="14" customFormat="1" ht="19.5" customHeight="1">
+      <c r="A11" s="15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:13" s="24" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A12" s="21" t="s">
+    <row r="12" spans="1:13" s="17" customFormat="1" ht="17.25" customHeight="1">
+      <c r="A12" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="23"/>
-      <c r="J12" s="25"/>
-    </row>
-    <row r="13" spans="1:13" s="9" customFormat="1" ht="18" customHeight="1">
-      <c r="A13" s="20" t="s">
+      <c r="B12" s="16"/>
+      <c r="J12" s="18"/>
+    </row>
+    <row r="13" spans="1:13" s="7" customFormat="1" ht="18" customHeight="1">
+      <c r="A13" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="11"/>
-      <c r="M13" s="36"/>
-    </row>
-    <row r="14" spans="1:13" s="33" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A14" s="51" t="s">
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="9"/>
+      <c r="M13" s="22"/>
+    </row>
+    <row r="14" spans="1:13" s="19" customFormat="1" ht="18.75" customHeight="1">
+      <c r="A14" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="51" t="s">
+      <c r="B14" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="56" t="s">
+      <c r="C14" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="56" t="s">
+      <c r="D14" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="52" t="s">
+      <c r="E14" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="53"/>
-      <c r="G14" s="58" t="s">
+      <c r="F14" s="34"/>
+      <c r="G14" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="58"/>
-      <c r="I14" s="54" t="s">
+      <c r="H14" s="39"/>
+      <c r="I14" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="55"/>
-      <c r="K14" s="54" t="s">
+      <c r="J14" s="36"/>
+      <c r="K14" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="L14" s="55"/>
-      <c r="M14" s="49" t="s">
+      <c r="L14" s="36"/>
+      <c r="M14" s="30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:13" s="33" customFormat="1" ht="33">
-      <c r="A15" s="50"/>
-      <c r="B15" s="50"/>
-      <c r="C15" s="57"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="35" t="s">
+    <row r="15" spans="1:13" s="19" customFormat="1" ht="33">
+      <c r="A15" s="31"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="34" t="s">
+      <c r="F15" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="35" t="s">
+      <c r="G15" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="H15" s="34" t="s">
+      <c r="H15" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="I15" s="35" t="s">
+      <c r="I15" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="J15" s="34" t="s">
+      <c r="J15" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="K15" s="35" t="s">
+      <c r="K15" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="L15" s="34" t="s">
+      <c r="L15" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="M15" s="50"/>
+      <c r="M15" s="31"/>
     </row>
     <row r="16" spans="1:13" s="1" customFormat="1" ht="18.75" customHeight="1">
       <c r="A16" s="3"/>
@@ -1434,152 +1334,225 @@
       <c r="M22" s="2"/>
     </row>
     <row r="23" spans="1:13" s="1" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
+      <c r="A23" s="40"/>
+      <c r="B23" s="40"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="40"/>
+      <c r="I23" s="40"/>
+      <c r="J23" s="40"/>
+      <c r="K23" s="40"/>
+      <c r="L23" s="40"/>
+      <c r="M23" s="40"/>
     </row>
     <row r="24" spans="1:13" s="1" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="6"/>
-      <c r="M24" s="6"/>
-    </row>
-    <row r="25" spans="1:13" s="8" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A25" s="47" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" s="48"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="17"/>
-      <c r="M25" s="17"/>
-    </row>
-    <row r="26" spans="1:13" s="28" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A26" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="27"/>
-      <c r="K26" s="27"/>
-      <c r="L26" s="27"/>
-      <c r="M26" s="27"/>
-    </row>
-    <row r="27" spans="1:13" s="28" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A27" s="29"/>
-      <c r="B27" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="39"/>
-      <c r="I27" s="39"/>
-      <c r="J27" s="39"/>
-      <c r="K27" s="39"/>
-      <c r="L27" s="39"/>
-      <c r="M27" s="30"/>
-    </row>
-    <row r="28" spans="1:13" s="28" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A28" s="29"/>
-      <c r="B28" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="32"/>
-      <c r="J28" s="32"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="30"/>
-    </row>
-    <row r="29" spans="1:13" s="41" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A29" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="C29" s="41" t="s">
-        <v>29</v>
-      </c>
-      <c r="F29" s="42"/>
-      <c r="G29" s="42" t="s">
-        <v>30</v>
-      </c>
-      <c r="H29" s="42"/>
-      <c r="I29" s="42"/>
-      <c r="L29" s="41" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" s="18" customFormat="1" ht="22.5" customHeight="1">
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="13"/>
-      <c r="K30" s="13"/>
-      <c r="M30" s="13"/>
-    </row>
-    <row r="31" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="32" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="33" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="34" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="35" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="36" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="37" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="38" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="39" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="40" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="41" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="42" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="43" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="44" s="1" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="45" s="1" customFormat="1" ht="22.5" customHeight="1"/>
+      <c r="A24" s="41"/>
+      <c r="B24" s="41"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="41"/>
+      <c r="K24" s="41"/>
+      <c r="L24" s="41"/>
+      <c r="M24" s="41"/>
+    </row>
+    <row r="25" spans="1:13" s="11" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A25" s="42"/>
+      <c r="B25" s="42"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="43"/>
+      <c r="I25" s="43"/>
+      <c r="J25" s="44"/>
+      <c r="K25" s="44"/>
+      <c r="L25" s="42"/>
+      <c r="M25" s="44"/>
+    </row>
+    <row r="26" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A26" s="41"/>
+      <c r="B26" s="41"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="41"/>
+      <c r="H26" s="41"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="41"/>
+      <c r="K26" s="41"/>
+      <c r="L26" s="41"/>
+      <c r="M26" s="41"/>
+    </row>
+    <row r="27" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A27" s="41"/>
+      <c r="B27" s="41"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="41"/>
+      <c r="F27" s="41"/>
+      <c r="G27" s="41"/>
+      <c r="H27" s="41"/>
+      <c r="I27" s="41"/>
+      <c r="J27" s="41"/>
+      <c r="K27" s="41"/>
+      <c r="L27" s="41"/>
+      <c r="M27" s="41"/>
+    </row>
+    <row r="28" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A28" s="41"/>
+      <c r="B28" s="41"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="41"/>
+      <c r="F28" s="41"/>
+      <c r="G28" s="41"/>
+      <c r="H28" s="41"/>
+      <c r="I28" s="41"/>
+      <c r="J28" s="41"/>
+      <c r="K28" s="41"/>
+      <c r="L28" s="41"/>
+      <c r="M28" s="41"/>
+    </row>
+    <row r="29" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A29" s="41"/>
+      <c r="B29" s="41"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="41"/>
+      <c r="F29" s="41"/>
+      <c r="G29" s="41"/>
+      <c r="H29" s="41"/>
+      <c r="I29" s="41"/>
+      <c r="J29" s="41"/>
+      <c r="K29" s="41"/>
+      <c r="L29" s="41"/>
+      <c r="M29" s="41"/>
+    </row>
+    <row r="30" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A30" s="41"/>
+      <c r="B30" s="41"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="41"/>
+      <c r="I30" s="41"/>
+      <c r="J30" s="41"/>
+      <c r="K30" s="41"/>
+      <c r="L30" s="41"/>
+      <c r="M30" s="41"/>
+    </row>
+    <row r="31" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A31" s="41"/>
+      <c r="B31" s="41"/>
+      <c r="C31" s="41"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="41"/>
+      <c r="F31" s="41"/>
+      <c r="G31" s="41"/>
+      <c r="H31" s="41"/>
+      <c r="I31" s="41"/>
+      <c r="J31" s="41"/>
+      <c r="K31" s="41"/>
+      <c r="L31" s="41"/>
+      <c r="M31" s="41"/>
+    </row>
+    <row r="32" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A32" s="41"/>
+      <c r="B32" s="41"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="41"/>
+      <c r="H32" s="41"/>
+      <c r="I32" s="41"/>
+      <c r="J32" s="41"/>
+      <c r="K32" s="41"/>
+      <c r="L32" s="41"/>
+      <c r="M32" s="41"/>
+    </row>
+    <row r="33" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A33" s="41"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+    </row>
+    <row r="34" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A34" s="41"/>
+      <c r="B34" s="41"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="41"/>
+      <c r="F34" s="41"/>
+      <c r="G34" s="41"/>
+      <c r="H34" s="41"/>
+      <c r="I34" s="41"/>
+      <c r="J34" s="41"/>
+      <c r="K34" s="41"/>
+      <c r="L34" s="41"/>
+      <c r="M34" s="41"/>
+    </row>
+    <row r="35" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A35" s="41"/>
+      <c r="B35" s="41"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="41"/>
+      <c r="F35" s="41"/>
+      <c r="G35" s="41"/>
+      <c r="H35" s="41"/>
+      <c r="I35" s="41"/>
+      <c r="J35" s="41"/>
+      <c r="K35" s="41"/>
+      <c r="L35" s="41"/>
+      <c r="M35" s="41"/>
+    </row>
+    <row r="36" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A36" s="41"/>
+      <c r="B36" s="41"/>
+      <c r="C36" s="41"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="41"/>
+      <c r="F36" s="41"/>
+      <c r="G36" s="41"/>
+      <c r="H36" s="41"/>
+      <c r="I36" s="41"/>
+      <c r="J36" s="41"/>
+      <c r="K36" s="41"/>
+      <c r="L36" s="41"/>
+      <c r="M36" s="41"/>
+    </row>
+    <row r="37" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1"/>
+    <row r="38" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1"/>
+    <row r="39" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1"/>
+    <row r="40" spans="1:13" s="1" customFormat="1" ht="22.5" customHeight="1"/>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="15">
     <mergeCell ref="A7:M7"/>
     <mergeCell ref="A5:M5"/>
     <mergeCell ref="A6:M6"/>
     <mergeCell ref="L2:M2"/>
-    <mergeCell ref="A25:B25"/>
     <mergeCell ref="M14:M15"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="B14:B15"/>
@@ -1654,38 +1627,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="37731f6e-0f2d-4bf4-b84c-108a697c7149">JSJPMY3Q7F3Z-1705263219-56</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="37731f6e-0f2d-4bf4-b84c-108a697c7149">
-      <Url>https://eoffice.hoaphat.com.vn/record25/dungquat/_layouts/15/DocIdRedir.aspx?ID=JSJPMY3Q7F3Z-1705263219-56</Url>
-      <Description>JSJPMY3Q7F3Z-1705263219-56</Description>
-    </_dlc_DocIdUrl>
-    <WorkflowID xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
-    <DocumentCategory xmlns="9091d8c9-259b-4840-8645-993eadbb66f9">434;#Tài liệu tham khảo</DocumentCategory>
-    <Required xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
-    <Abstract xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
-    <WorkflowURL xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
-    <Workflow xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
-    <RequestCode xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
-    <DocumentCategoryData xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
-    <DocumentCategoryID xmlns="9091d8c9-259b-4840-8645-993eadbb66f9">434</DocumentCategoryID>
-    <Index xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
-    <WorkflowStatus xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100685DE914C0E1EF419246CB56320D150C" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fd91d82f5c365423259a479c28de9e14">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="37731f6e-0f2d-4bf4-b84c-108a697c7149" xmlns:ns3="9091d8c9-259b-4840-8645-993eadbb66f9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a4415d62f5572c90b77cb9ba30664b0c" ns2:_="" ns3:_="">
     <xsd:import namespace="37731f6e-0f2d-4bf4-b84c-108a697c7149"/>
@@ -1907,6 +1848,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="37731f6e-0f2d-4bf4-b84c-108a697c7149">JSJPMY3Q7F3Z-1705263219-56</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="37731f6e-0f2d-4bf4-b84c-108a697c7149">
+      <Url>https://eoffice.hoaphat.com.vn/record25/dungquat/_layouts/15/DocIdRedir.aspx?ID=JSJPMY3Q7F3Z-1705263219-56</Url>
+      <Description>JSJPMY3Q7F3Z-1705263219-56</Description>
+    </_dlc_DocIdUrl>
+    <WorkflowID xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
+    <DocumentCategory xmlns="9091d8c9-259b-4840-8645-993eadbb66f9">434;#Tài liệu tham khảo</DocumentCategory>
+    <Required xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
+    <Abstract xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
+    <WorkflowURL xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
+    <Workflow xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
+    <RequestCode xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
+    <DocumentCategoryData xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
+    <DocumentCategoryID xmlns="9091d8c9-259b-4840-8645-993eadbb66f9">434</DocumentCategoryID>
+    <Index xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
+    <WorkflowStatus xmlns="9091d8c9-259b-4840-8645-993eadbb66f9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E20EF549-B0B6-47F9-994B-D6C7C1DA2558}">
   <ds:schemaRefs>
@@ -1916,9 +1889,20 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36F4CF3A-0058-409C-BCCA-0B5CB7058448}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CB90150D-CCB7-4704-AF5F-696F6BED57EF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="37731f6e-0f2d-4bf4-b84c-108a697c7149"/>
+    <ds:schemaRef ds:uri="9091d8c9-259b-4840-8645-993eadbb66f9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1935,20 +1919,9 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CB90150D-CCB7-4704-AF5F-696F6BED57EF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36F4CF3A-0058-409C-BCCA-0B5CB7058448}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="37731f6e-0f2d-4bf4-b84c-108a697c7149"/>
-    <ds:schemaRef ds:uri="9091d8c9-259b-4840-8645-993eadbb66f9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>